<commit_message>
Review fixes: harden calc core, unique email, security headers, demo derives figures from data
- calc: validate dates (throw instead of NaN), round money to fils, guard zero/negative demand
- schema: unique index on lower(email) (migration 0001) so bootstrap cannot create duplicates
- headers: nosniff, frame deny, referrer, permissions, HSTS; noindex
- demo: overdue days from due dates, expiry loss/profit/standalone sales derived, margin constant
- tests: demo-vs-core consistency (jsdom), edge cases
- workbook: relabel project-vs-category target row as illustration

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/Sadaf_inputs_workbook.xlsx
+++ b/docs/Sadaf_inputs_workbook.xlsx
@@ -7987,7 +7987,7 @@
     </x:row>
     <x:row r="53" ht="34" customHeight="1">
       <x:c r="A53" s="33" t="str">
-        <x:v>Sales versus target</x:v>
+        <x:v>Project sales as share of category target (illustration only)</x:v>
       </x:c>
       <x:c r="B53" s="37" t="n">
         <x:f>IF(B52=0,"No target",B41/B52)</x:f>
@@ -7998,7 +7998,9 @@
         <x:v>0.9375</x:v>
       </x:c>
       <x:c r="D53" s="2"/>
-      <x:c r="E53" s="39"/>
+      <x:c r="E53" s="39" t="str">
+        <x:v>One project against a whole category monthly target, so this is not target attainment. Real attainment = all sales of the SAME category and month / that target (calc.ts: attainment).</x:v>
+      </x:c>
     </x:row>
     <x:row r="54" ht="34" customHeight="1">
       <x:c r="A54" s="33"/>

</xml_diff>

<commit_message>
Sales import reads an optional due date; update inputs workbook for importer and estimates
- E03 sales files may carry a contractual due date per invoice. It is stored
  on the invoice (a later unpaid-invoice file without one does not erase it),
  rejected if before the invoice date, and the reconciliation summary counts
  invoices without one. Needed to measure payment lateness for invoices that
  are paid before the first unpaid-invoice snapshot.
- docs/Sadaf_inputs_workbook.xlsx (edited at package level, so all other sheets
  are byte-identical): "Start here" B20/B21 describe the importer; ERP
  requirements E03/E04 gain the due-date and invoice-link requirements; new
  sheet "Imports and predictions" (import rules, columns read per file type,
  estimate features with minimum history, history to load).
- START_HERE.md notes the workbook is no longer identical to the archived copy.

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/Sadaf_inputs_workbook.xlsx
+++ b/docs/Sadaf_inputs_workbook.xlsx
@@ -6,6 +6,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Start here" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Report map" sheetId="2" state="visible" r:id="rId2"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ERP requirements" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Imports and predictions" sheetId="10" state="visible" r:id="rId12"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Basic weekly" sheetId="4" state="visible" r:id="rId4"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Basic monthly" sheetId="5" state="visible" r:id="rId5"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Advanced weekly" sheetId="6" state="visible" r:id="rId6"/>
@@ -1136,7 +1137,7 @@
       </c>
       <c r="B20" s="10" t="inlineStr">
         <is>
-          <t>The reviewed site displays fixed demo data. Its upload feature checks CSV columns/values; it does not load this workbook or regenerate real reports.</t>
+          <t>There are two sites. The demo site shows fixed synthetic data and does not load this workbook. The main app lets the company owner import CSV exports of E01–E07 and the installed-equipment list on its Import data page (see sheet 'Imports and predictions'). The dashboard does not yet read imported data.</t>
         </is>
       </c>
     </row>
@@ -1148,7 +1149,7 @@
       </c>
       <c r="B21" s="11" t="inlineStr">
         <is>
-          <t>Connect the confirmed Alpha exports and these manual tables, calculate the reports, and reconcile totals. This workbook is the data checklist and entry guide.</t>
+          <t>Connect the confirmed Alpha exports and these manual tables, calculate the reports, and reconcile totals. The CSV importer and the estimate calculations are built; the report screens that use imported data, XLSX upload and the manual-table forms are still to build. This workbook is the data checklist and entry guide.</t>
         </is>
       </c>
     </row>
@@ -1333,6 +1334,664 @@
   <tableParts count="1">
     <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
   </tableParts>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <tabColor rgb="FF176E60"/>
+  </sheetPr>
+  <dimension ref="A1:F39"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="28" customWidth="1" min="1" max="1"/>
+    <col width="52" customWidth="1" min="2" max="2"/>
+    <col width="52" customWidth="1" min="3" max="3"/>
+    <col width="30" customWidth="1" min="4" max="4"/>
+    <col width="52" customWidth="1" min="5" max="5"/>
+    <col width="42" customWidth="1" min="6" max="6"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="24" customHeight="1"/>
+    <row r="2" ht="33" customHeight="1">
+      <c r="A2" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Importing data and the estimate features (v7)</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="12" customHeight="1"/>
+    <row r="4" ht="24" customHeight="1">
+      <c r="A4" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">How the app loads the Alpha exports, and the data the new estimate features need.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="24" customHeight="1">
+      <c r="A5" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Header names are assumptions until a real Alpha export is checked. Estimates are labelled ESTIMATED and are never shown as facts.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="12" customHeight="1"/>
+    <row r="7" ht="26" customHeight="1">
+      <c r="A7" s="14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1. How importing works</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="30" customHeight="1">
+      <c r="A8" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Topic</t>
+        </is>
+      </c>
+      <c r="B8" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Rule</t>
+        </is>
+      </c>
+      <c r="C8" s="8" t="n"/>
+      <c r="D8" s="8" t="n"/>
+      <c r="E8" s="8" t="n"/>
+      <c r="F8" s="8" t="n"/>
+    </row>
+    <row r="9" ht="24" customHeight="1">
+      <c r="A9" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Who and where</t>
+        </is>
+      </c>
+      <c r="B9" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">The company owner uploads CSV files on the Import data page of the app: UTF-8, one file per type, up to 4.5 MB. Split large sales exports by month. In Excel use Save As, CSV UTF-8.</t>
+        </is>
+      </c>
+      <c r="C9" s="10" t="n"/>
+      <c r="D9" s="10" t="n"/>
+      <c r="E9" s="10" t="n"/>
+      <c r="F9" s="10" t="n"/>
+    </row>
+    <row r="10" ht="38" customHeight="1">
+      <c r="A10" s="11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Order</t>
+        </is>
+      </c>
+      <c r="B10" s="11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Import E01 products and E02 customers first, then E03 sales, E04 receipts, E05 unpaid invoices, E06 stock, E07 stock transactions and installed equipment. Later files point at product and customer codes that must already exist. A row with an unknown code is rejected; it is never created.</t>
+        </is>
+      </c>
+      <c r="C10" s="11" t="n"/>
+      <c r="D10" s="11" t="n"/>
+      <c r="E10" s="11" t="n"/>
+      <c r="F10" s="11" t="n"/>
+    </row>
+    <row r="11" ht="24" customHeight="1">
+      <c r="A11" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Check first</t>
+        </is>
+      </c>
+      <c r="B11" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Use Check file before Import. It validates every row and shows totals (net sales, cash received, outstanding by age, stock value) to compare with Alpha, and saves nothing.</t>
+        </is>
+      </c>
+      <c r="C11" s="10" t="n"/>
+      <c r="D11" s="10" t="n"/>
+      <c r="E11" s="10" t="n"/>
+      <c r="F11" s="10" t="n"/>
+    </row>
+    <row r="12" ht="24" customHeight="1">
+      <c r="A12" s="11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">No double counting</t>
+        </is>
+      </c>
+      <c r="B12" s="11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">The same file cannot be imported twice. A changed file updates rows by their ERP IDs (invoice + line, receipt + allocation row, transaction ID, product / customer / unit codes); it never duplicates them.</t>
+        </is>
+      </c>
+      <c r="C12" s="11" t="n"/>
+      <c r="D12" s="11" t="n"/>
+      <c r="E12" s="11" t="n"/>
+      <c r="F12" s="11" t="n"/>
+    </row>
+    <row r="13" ht="38" customHeight="1">
+      <c r="A13" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Snapshot files</t>
+        </is>
+      </c>
+      <c r="B13" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Unpaid invoices (E05) and stock by batch (E06) are point-in-time. A file for a date replaces that date; other dates are kept and never added together. The file needs a snapshot date column, or the date is entered when uploading.</t>
+        </is>
+      </c>
+      <c r="C13" s="10" t="n"/>
+      <c r="D13" s="10" t="n"/>
+      <c r="E13" s="10" t="n"/>
+      <c r="F13" s="10" t="n"/>
+    </row>
+    <row r="14" ht="24" customHeight="1">
+      <c r="A14" s="11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Bad rows</t>
+        </is>
+      </c>
+      <c r="B14" s="11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Good rows are saved and bad rows are listed with the row number and the reason (status Partial). Fix them in the file and import it again.</t>
+        </is>
+      </c>
+      <c r="C14" s="11" t="n"/>
+      <c r="D14" s="11" t="n"/>
+      <c r="E14" s="11" t="n"/>
+      <c r="F14" s="11" t="n"/>
+    </row>
+    <row r="15" ht="38" customHeight="1">
+      <c r="A15" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Unknown stays unknown</t>
+        </is>
+      </c>
+      <c r="B15" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">A blank due date, cost, segment, credit limit or payment term is kept as unknown, never as 0 or a default segment. An unrecognised customer segment is left unclassified with a warning. Public / government / tender wording is read as Tender.</t>
+        </is>
+      </c>
+      <c r="C15" s="10" t="n"/>
+      <c r="D15" s="10" t="n"/>
+      <c r="E15" s="10" t="n"/>
+      <c r="F15" s="10" t="n"/>
+    </row>
+    <row r="16" ht="38" customHeight="1">
+      <c r="A16" s="11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Dates and numbers</t>
+        </is>
+      </c>
+      <c r="B16" s="11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Dates as YYYY-MM-DD or day-first D/M/YYYY; month-first dates are not supported. Dates after the import day are rejected. Amounts are JOD with a decimal point; returns are negative; thousands separators are accepted. Arabic text and Arabic digits are accepted.</t>
+        </is>
+      </c>
+      <c r="C16" s="11" t="n"/>
+      <c r="D16" s="11" t="n"/>
+      <c r="E16" s="11" t="n"/>
+      <c r="F16" s="11" t="n"/>
+    </row>
+    <row r="17" ht="24" customHeight="1">
+      <c r="A17" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Receipts</t>
+        </is>
+      </c>
+      <c r="B17" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">If the file has a receipt total column, the allocation rows of a receipt must add up to it. An allocation to an invoice that is not in the imported invoices is kept once, as not linked to an invoice, with a warning.</t>
+        </is>
+      </c>
+      <c r="C17" s="10" t="n"/>
+      <c r="D17" s="10" t="n"/>
+      <c r="E17" s="10" t="n"/>
+      <c r="F17" s="10" t="n"/>
+    </row>
+    <row r="18" ht="24" customHeight="1">
+      <c r="A18" s="11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Column names</t>
+        </is>
+      </c>
+      <c r="B18" s="11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">The header names below are assumptions, not Alpha's real column names. Matching ignores case, spaces and punctuation and accepts common alternatives. They are adjusted once a real Alpha export is checked.</t>
+        </is>
+      </c>
+      <c r="C18" s="11" t="n"/>
+      <c r="D18" s="11" t="n"/>
+      <c r="E18" s="11" t="n"/>
+      <c r="F18" s="11" t="n"/>
+    </row>
+    <row r="19" ht="12" customHeight="1"/>
+    <row r="20" ht="26" customHeight="1">
+      <c r="A20" s="14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2. Columns the importer reads (first name shown; other spellings are accepted)</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="30" customHeight="1">
+      <c r="A21" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">File type</t>
+        </is>
+      </c>
+      <c r="B21" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Required columns</t>
+        </is>
+      </c>
+      <c r="C21" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Optional columns</t>
+        </is>
+      </c>
+      <c r="D21" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Point in time?</t>
+        </is>
+      </c>
+      <c r="E21" s="8" t="n"/>
+      <c r="F21" s="8" t="n"/>
+    </row>
+    <row r="22" ht="38" customHeight="1">
+      <c r="A22" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Product and supplier list (E01)</t>
+        </is>
+      </c>
+      <c r="B22" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">product code, product name, category</t>
+        </is>
+      </c>
+      <c r="C22" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">manufacturer, supplier code, supplier name, unit, pack conversion, expiry tracked, active</t>
+        </is>
+      </c>
+      <c r="D22" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">No</t>
+        </is>
+      </c>
+      <c r="E22" s="10" t="n"/>
+      <c r="F22" s="10" t="n"/>
+    </row>
+    <row r="23" ht="38" customHeight="1">
+      <c r="A23" s="11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Customer list (E02)</t>
+        </is>
+      </c>
+      <c r="B23" s="11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">customer code, customer name</t>
+        </is>
+      </c>
+      <c r="C23" s="11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">city, customer type, segment, payment terms, credit limit, account owner, active</t>
+        </is>
+      </c>
+      <c r="D23" s="11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">No</t>
+        </is>
+      </c>
+      <c r="E23" s="11" t="n"/>
+      <c r="F23" s="11" t="n"/>
+    </row>
+    <row r="24" ht="38" customHeight="1">
+      <c r="A24" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Sales and returns (E03)</t>
+        </is>
+      </c>
+      <c r="B24" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">invoice no, line no, invoice date, customer code, product code, quantity, net sales</t>
+        </is>
+      </c>
+      <c r="C24" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">due date, doc type, product cost, project, account owner</t>
+        </is>
+      </c>
+      <c r="D24" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">No</t>
+        </is>
+      </c>
+      <c r="E24" s="10" t="n"/>
+      <c r="F24" s="10" t="n"/>
+    </row>
+    <row r="25" ht="38" customHeight="1">
+      <c r="A25" s="11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Customer receipts (E04)</t>
+        </is>
+      </c>
+      <c r="B25" s="11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">receipt no, allocation row id, receipt date, customer code, allocated amount</t>
+        </is>
+      </c>
+      <c r="C25" s="11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">invoice no, receipt total</t>
+        </is>
+      </c>
+      <c r="D25" s="11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">No</t>
+        </is>
+      </c>
+      <c r="E25" s="11" t="n"/>
+      <c r="F25" s="11" t="n"/>
+    </row>
+    <row r="26" ht="38" customHeight="1">
+      <c r="A26" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Unpaid invoices (E05)</t>
+        </is>
+      </c>
+      <c r="B26" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">invoice no, customer code, invoice date, remaining amount</t>
+        </is>
+      </c>
+      <c r="C26" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">snapshot date, due date, account owner</t>
+        </is>
+      </c>
+      <c r="D26" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Yes: needs a snapshot date (column or upload form)</t>
+        </is>
+      </c>
+      <c r="E26" s="10" t="n"/>
+      <c r="F26" s="10" t="n"/>
+    </row>
+    <row r="27" ht="38" customHeight="1">
+      <c r="A27" s="11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Stock by batch (E06)</t>
+        </is>
+      </c>
+      <c r="B27" s="11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">product code, warehouse, quantity</t>
+        </is>
+      </c>
+      <c r="C27" s="11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">snapshot date, batch, unit cost, expiry date, owned</t>
+        </is>
+      </c>
+      <c r="D27" s="11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Yes: needs a snapshot date (column or upload form)</t>
+        </is>
+      </c>
+      <c r="E27" s="11" t="n"/>
+      <c r="F27" s="11" t="n"/>
+    </row>
+    <row r="28" ht="38" customHeight="1">
+      <c r="A28" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Stock transactions (E07)</t>
+        </is>
+      </c>
+      <c r="B28" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">transaction id, transaction date, product code, warehouse, transaction type, quantity</t>
+        </is>
+      </c>
+      <c r="C28" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">batch</t>
+        </is>
+      </c>
+      <c r="D28" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">No</t>
+        </is>
+      </c>
+      <c r="E28" s="10" t="n"/>
+      <c r="F28" s="10" t="n"/>
+    </row>
+    <row r="29" ht="38" customHeight="1">
+      <c r="A29" s="11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Installed equipment (E11 or manual)</t>
+        </is>
+      </c>
+      <c r="B29" s="11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">unit code, customer code, unit name</t>
+        </is>
+      </c>
+      <c r="C29" s="11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">product code, installed on, warranty end, service, expected monthly consumables</t>
+        </is>
+      </c>
+      <c r="D29" s="11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">No</t>
+        </is>
+      </c>
+      <c r="E29" s="11" t="n"/>
+      <c r="F29" s="11" t="n"/>
+    </row>
+    <row r="30" ht="12" customHeight="1"/>
+    <row r="31" ht="26" customHeight="1">
+      <c r="A31" s="14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">3. Estimate features (calculations are built and tested; the screens that show them are not built yet)</t>
+        </is>
+      </c>
+    </row>
+    <row r="32" ht="30" customHeight="1">
+      <c r="A32" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Feature</t>
+        </is>
+      </c>
+      <c r="B32" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Question it answers</t>
+        </is>
+      </c>
+      <c r="C32" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Data needed</t>
+        </is>
+      </c>
+      <c r="D32" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Minimum history</t>
+        </is>
+      </c>
+      <c r="E32" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Shown as</t>
+        </is>
+      </c>
+      <c r="F32" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">If data is missing</t>
+        </is>
+      </c>
+    </row>
+    <row r="33" ht="68" customHeight="1">
+      <c r="A33" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Repurchase timing</t>
+        </is>
+      </c>
+      <c r="B33" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Which customers are due, overdue or lapsed on reordering?</t>
+        </is>
+      </c>
+      <c r="C33" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">E03 order dates per customer.</t>
+        </is>
+      </c>
+      <c r="D33" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">At least 4 distinct order dates per customer.</t>
+        </is>
+      </c>
+      <c r="E33" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ESTIMATED. Typical days between orders (median), expected next order date, level On cycle / Due soon / Overdue / Lapsed, and confidence Higher or Lower when the intervals vary a lot.</t>
+        </is>
+      </c>
+      <c r="F33" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">'Not enough data'. Nothing is guessed. An order dated after the report date is treated as a bad import.</t>
+        </is>
+      </c>
+    </row>
+    <row r="34" ht="53" customHeight="1">
+      <c r="A34" s="11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Payment behaviour</t>
+        </is>
+      </c>
+      <c r="B34" s="11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">How late does each customer usually pay?</t>
+        </is>
+      </c>
+      <c r="C34" s="11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Invoice due date (E03 due date or E05) and payment date (E04 receipt allocated to that invoice).</t>
+        </is>
+      </c>
+      <c r="D34" s="11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">At least 5 paid invoices per customer.</t>
+        </is>
+      </c>
+      <c r="E34" s="11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ESTIMATED. Typical days late (median), a cautious figure that 80% of invoices stay within, and the share of invoices paid late.</t>
+        </is>
+      </c>
+      <c r="F34" s="11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">'Not enough data'. Invoices without a due date or without an invoice link on the receipt do not count.</t>
+        </is>
+      </c>
+    </row>
+    <row r="35" ht="83" customHeight="1">
+      <c r="A35" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Cash forecast</t>
+        </is>
+      </c>
+      <c r="B35" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">How much cash is likely in the next 30 / 60 / 90 days?</t>
+        </is>
+      </c>
+      <c r="C35" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">E05 unpaid invoices plus each customer's payment behaviour.</t>
+        </is>
+      </c>
+      <c r="D35" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Customers with enough payment history (see above).</t>
+        </is>
+      </c>
+      <c r="E35" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ESTIMATED. Expected collections per window. Invoices already past their customer's typical payment day, invoices of customers without history, and invoices expected after 90 days are shown separately.</t>
+        </is>
+      </c>
+      <c r="F35" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Money that cannot be forecast is listed, not guessed. The parts always add up to the total outstanding.</t>
+        </is>
+      </c>
+    </row>
+    <row r="36" ht="53" customHeight="1">
+      <c r="A36" s="11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Opportunity ranking</t>
+        </is>
+      </c>
+      <c r="B36" s="11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Which customers should the team call first?</t>
+        </is>
+      </c>
+      <c r="C36" s="11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">The signals above (for example overdue repurchase) and the consumables purchase gap, each with an estimated JOD value.</t>
+        </is>
+      </c>
+      <c r="D36" s="11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Not applicable.</t>
+        </is>
+      </c>
+      <c r="E36" s="11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ESTIMATED. One line per customer showing the largest signal; other signals on the same customer are named but not added.</t>
+        </is>
+      </c>
+      <c r="F36" s="11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Only signals with a positive value are ranked. The total is not the sum of overlapping signals.</t>
+        </is>
+      </c>
+    </row>
+    <row r="37" ht="12" customHeight="1"/>
+    <row r="38" ht="26" customHeight="1">
+      <c r="A38" s="14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">4. History to load before the first use</t>
+        </is>
+      </c>
+    </row>
+    <row r="39" ht="38" customHeight="1">
+      <c r="A39" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Minimum to start</t>
+        </is>
+      </c>
+      <c r="B39" s="10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Load all available history, ideally 12 months: E03 sales with order dates and due dates, and E04 receipts linked to their invoices. Then keep adding E03, E04 and E05 weekly. A customer who orders monthly needs about 4 months of orders and 5 paid invoices before an estimate appears; until then the feature says 'Not enough data'.</t>
+        </is>
+      </c>
+      <c r="C39" s="10" t="n"/>
+      <c r="D39" s="10" t="n"/>
+      <c r="E39" s="10" t="n"/>
+      <c r="F39" s="10" t="n"/>
+    </row>
+  </sheetData>
+  <mergeCells count="12">
+    <mergeCell ref="B8:F8"/>
+    <mergeCell ref="B9:F9"/>
+    <mergeCell ref="B10:F10"/>
+    <mergeCell ref="B11:F11"/>
+    <mergeCell ref="B12:F12"/>
+    <mergeCell ref="B13:F13"/>
+    <mergeCell ref="B14:F14"/>
+    <mergeCell ref="B15:F15"/>
+    <mergeCell ref="B16:F16"/>
+    <mergeCell ref="B17:F17"/>
+    <mergeCell ref="B18:F18"/>
+    <mergeCell ref="B39:F39"/>
+  </mergeCells>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
@@ -2654,7 +3313,7 @@
       </c>
       <c r="D11" s="10" t="inlineStr">
         <is>
-          <t>Invoice and line IDs; date/type; customer; product; signed quantity, net sales and product cost JOD excluding tax. Project/order link is required for project profit; unit link when available. Keep returns/credits. Also export the same lines for the same months of the previous year (growth against last year).</t>
+          <t>Invoice and line IDs; date/type; customer; product; signed quantity, net sales and product cost JOD excluding tax. Project/order link is required for project profit; unit link when available. Keep returns/credits. Also export the same lines for the same months of the previous year (growth against last year). Add the contractual due date of each invoice where the ERP has it: it is needed to measure how late each customer pays, and E05 carries it only while the invoice is unpaid.</t>
         </is>
       </c>
       <c r="E11" s="10" t="inlineStr">
@@ -2692,7 +3351,7 @@
       </c>
       <c r="D12" s="11" t="inlineStr">
         <is>
-          <t>Receipt ID; allocation row ID; receipt date; customer; invoice/line link where available; allocated JOD. Include unapplied cash once. Allocation rows must add to the receipt total.</t>
+          <t>Receipt ID; allocation row ID; receipt date; customer; invoice/line link where available; allocated JOD. Include unapplied cash once. Allocation rows must add to the receipt total. Link each allocation to its invoice wherever possible: without the link, payment lateness cannot be measured.</t>
         </is>
       </c>
       <c r="E12" s="11" t="inlineStr">

</xml_diff>

<commit_message>
Products carry an optional therapeutic area (column, import field, workbook)
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/Sadaf_inputs_workbook.xlsx
+++ b/docs/Sadaf_inputs_workbook.xlsx
@@ -1137,7 +1137,7 @@
       </c>
       <c r="B20" s="10" t="inlineStr">
         <is>
-          <t>There are two sites. The demo site shows fixed synthetic data and does not load this workbook. The main app lets the company owner import CSV exports of E01–E07 and the installed-equipment list on its Import data page (see sheet 'Imports and predictions'). The dashboard does not yet read imported data.</t>
+          <t>There are two sites. The demo site shows fixed synthetic data and does not load this workbook. The main app lets the company owner import CSV exports of E01–E07 and the installed-equipment list on its Import data page (see sheet 'Imports and predictions'). The Overview, Finance, Inventory, Management actions and Weekly summary screens read the imported data.</t>
         </is>
       </c>
     </row>
@@ -1149,7 +1149,7 @@
       </c>
       <c r="B21" s="11" t="inlineStr">
         <is>
-          <t>Connect the confirmed Alpha exports and these manual tables, calculate the reports, and reconcile totals. The CSV importer and the estimate calculations are built; the report screens that use imported data, XLSX upload and the manual-table forms are still to build. This workbook is the data checklist and entry guide.</t>
+          <t>Connect the confirmed Alpha exports and these manual tables, calculate the reports, and reconcile totals. The CSV importer, the report screens that use imported data and the estimate calculations are built; XLSX upload, the manual-table forms and the portfolio-growth view are still to build. This workbook is the data checklist and entry guide.</t>
         </is>
       </c>
     </row>
@@ -1592,7 +1592,7 @@
       <c r="E21" s="8" t="n"/>
       <c r="F21" s="8" t="n"/>
     </row>
-    <row r="22" ht="38" customHeight="1">
+    <row r="22" ht="53" customHeight="1">
       <c r="A22" s="10" t="inlineStr">
         <is>
           <t xml:space="preserve">Product and supplier list (E01)</t>
@@ -1605,7 +1605,7 @@
       </c>
       <c r="C22" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">manufacturer, supplier code, supplier name, unit, pack conversion, expiry tracked, active</t>
+          <t xml:space="preserve">therapeutic area, manufacturer, supplier code, supplier name, unit, pack conversion, expiry tracked, active</t>
         </is>
       </c>
       <c r="D22" s="10" t="inlineStr">
@@ -1788,7 +1788,7 @@
     <row r="31" ht="26" customHeight="1">
       <c r="A31" s="14" t="inlineStr">
         <is>
-          <t xml:space="preserve">3. Estimate features (calculations are built and tested; the screens that show them are not built yet)</t>
+          <t xml:space="preserve">3. Estimate features (built, tested and shown on the Management actions screen; each is labelled ESTIMATED)</t>
         </is>
       </c>
     </row>
@@ -3237,7 +3237,7 @@
       </c>
       <c r="D9" s="10" t="inlineStr">
         <is>
-          <t>Product code; product name; category (Equipment / Devices / Consumables); manufacturer; supplier code/name; counting unit; pack conversion; expiry tracked Yes/No.</t>
+          <t>Product code; product name; category (Equipment / Devices / Consumables); therapeutic area (optional, for example Respiratory or Critical care; used by the portfolio-growth view); manufacturer; supplier code/name; counting unit; pack conversion; expiry tracked Yes/No.</t>
         </is>
       </c>
       <c r="E9" s="10" t="inlineStr">

</xml_diff>